<commit_message>
feat: update products with Spanish details and local photos
Co-Authored-By: Oz <oz-agent@warp.dev>
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q65"/>
+  <dimension ref="A1:U65"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,6 +451,18 @@
       <c r="Q1" t="str">
         <v>is_published</v>
       </c>
+      <c r="R1" t="str">
+        <v>image_link_1</v>
+      </c>
+      <c r="S1" t="str">
+        <v>image_link_2</v>
+      </c>
+      <c r="T1" t="str">
+        <v>image_link_3</v>
+      </c>
+      <c r="U1" t="str">
+        <v>image_links</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -475,34 +487,46 @@
         <v>128GB</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>6.9" IPS LCD (HD+ 1600×720), hasta 120Hz</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>MediaTek Dimensity 6300 (6nm)</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + auxiliar; Frontal: 8MP</v>
       </c>
       <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
+        <v>6000mAh, 33W carga rápida</v>
+      </c>
+      <c r="M2">
+        <v>2025</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>Económico 5G teléfono con gran 6.9" 120Hz pantalla, Dimensity 6300 rendimiento, y a 6000mAh batería; incluye Xiaomi HyperOS.</v>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>/images/fotos/p-1.jpg</v>
       </c>
       <c r="P2" t="b">
         <v>0</v>
       </c>
       <c r="Q2" t="b">
         <v>1</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -528,34 +552,46 @@
         <v>128GB</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+ 2400×1080), 120Hz</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>MediaTek Helio G99-Ultra (6nm)</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>6GB</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>Trasera: 108MP + 2MP profundidad + 2MP macro; Frontal: 20MP</v>
       </c>
       <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
+        <v>5500mAh, 33W turbo carga</v>
+      </c>
+      <c r="M3">
+        <v>2024</v>
       </c>
       <c r="N3" t="str">
-        <v/>
+        <v>De gama media buena relación calidad-precio teléfono con 108MP sistema de cámaras, AMOLED 120Hz pantalla, Helio G99-Ultra chipset, y 5500mAh batería; Xiaomi HyperOS.</v>
       </c>
       <c r="O3" t="str">
-        <v/>
+        <v>/images/fotos/p-2.jpg</v>
       </c>
       <c r="P3" t="b">
         <v>0</v>
       </c>
       <c r="Q3" t="b">
         <v>1</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -581,34 +617,46 @@
         <v>64GB</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>6.88" IPS LCD (HD+), 120Hz</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>Unisoc T7250</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>Trasera: 32MP; Frontal: 8MP</v>
       </c>
       <c r="L4" t="str">
-        <v/>
-      </c>
-      <c r="M4" t="str">
-        <v/>
+        <v>5200mAh, 15W carga</v>
+      </c>
+      <c r="M4">
+        <v>2025</v>
       </c>
       <c r="N4" t="str">
-        <v/>
+        <v>De entrada teléfono con fluida 120Hz pantalla, Unisoc T7250, y a 5200mAh batería.</v>
       </c>
       <c r="O4" t="str">
-        <v/>
+        <v>/images/fotos/p-3.jpg</v>
       </c>
       <c r="P4" t="b">
         <v>0</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -634,34 +682,46 @@
         <v>32GB</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>6.52" IPS LCD (HD+ 1600×720)</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>MediaTek Helio G36 (12nm)</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>2GB</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>Trasera: 8MP + 0.08MP profundidad; Frontal: 5MP</v>
       </c>
       <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
-        <v/>
+        <v>5000mAh, 10W carga</v>
+      </c>
+      <c r="M5">
+        <v>2023</v>
       </c>
       <c r="N5" t="str">
-        <v/>
+        <v>De entrada Android (Go edition) teléfono con 6.52" pantalla, Helio G36 chipset, y 5000mAh batería.</v>
       </c>
       <c r="O5" t="str">
-        <v/>
+        <v>/images/fotos/p-4.jpg</v>
       </c>
       <c r="P5" t="b">
         <v>0</v>
       </c>
       <c r="Q5" t="b">
         <v>1</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -687,34 +747,46 @@
         <v>128GB</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>6.6" PLS LCD (FHD+ 2408×1080)</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>MediaTek Helio G80</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>Trasera: 50MP + 5MP ultra gran angular + 2MP macro; Frontal: 13MP</v>
       </c>
       <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
-        <v/>
+        <v>5000mAh, 15W carga</v>
+      </c>
+      <c r="M6">
+        <v>2023</v>
       </c>
       <c r="N6" t="str">
-        <v/>
+        <v>Económico Samsung teléfono con gran FHD+ pantalla, triple cámaras, y a 5000mAh batería.</v>
       </c>
       <c r="O6" t="str">
-        <v/>
+        <v>/images/fotos/p-5.webp</v>
       </c>
       <c r="P6" t="b">
         <v>0</v>
       </c>
       <c r="Q6" t="b">
         <v>1</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -740,34 +812,46 @@
         <v>128GB</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>6.1" Super Retina XDR OLED (2556×1179)</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>Apple A18</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>Trasera: 48MP Fusion + 12MP Ultra gran angular; Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L7" t="str">
-        <v/>
-      </c>
-      <c r="M7" t="str">
-        <v/>
+        <v>3561mAh (aprox.), carga rápida; MagSafe inalámbrica</v>
+      </c>
+      <c r="M7">
+        <v>2024</v>
       </c>
       <c r="N7" t="str">
-        <v/>
+        <v>Apple tope de gama con A18 chip, 6.1" OLED pantalla, y avanzado doble-sistema de cámaras con 48MP principal; es compatible con Apple Intelligence.</v>
       </c>
       <c r="O7" t="str">
-        <v/>
+        <v>/images/fotos/p-6.jpg</v>
       </c>
       <c r="P7" t="b">
         <v>0</v>
       </c>
       <c r="Q7" t="b">
         <v>1</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -793,34 +877,46 @@
         <v>128GB</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>6.88" IPS LCD (HD+), 120Hz</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>Unisoc T7250</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>Trasera: 32MP; Frontal: 8MP</v>
       </c>
       <c r="L8" t="str">
-        <v/>
-      </c>
-      <c r="M8" t="str">
-        <v/>
+        <v>5200mAh, 15W carga</v>
+      </c>
+      <c r="M8">
+        <v>2025</v>
       </c>
       <c r="N8" t="str">
-        <v/>
+        <v>De entrada teléfono con fluida 120Hz pantalla, Unisoc T7250, y a 5200mAh batería.</v>
       </c>
       <c r="O8" t="str">
-        <v/>
+        <v>/images/fotos/p-7.jpg</v>
       </c>
       <c r="P8" t="b">
         <v>0</v>
       </c>
       <c r="Q8" t="b">
         <v>1</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -846,34 +942,46 @@
         <v>128GB</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>6.7" PLS LCD (HD+ 720×1600)</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>MediaTek Helio G85 (12nm)</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K9" t="str">
-        <v/>
+        <v>Trasera: 50MP + 2MP profundidad; Frontal: 8MP</v>
       </c>
       <c r="L9" t="str">
-        <v/>
-      </c>
-      <c r="M9" t="str">
-        <v/>
+        <v>5000mAh, 25W carga</v>
+      </c>
+      <c r="M9">
+        <v>2024</v>
       </c>
       <c r="N9" t="str">
-        <v/>
+        <v>De entrada Samsung teléfono con gran 6.7" pantalla, Helio G85 rendimiento, y 5000mAh batería.</v>
       </c>
       <c r="O9" t="str">
-        <v/>
+        <v>/images/fotos/p-8.jpg</v>
       </c>
       <c r="P9" t="b">
         <v>0</v>
       </c>
       <c r="Q9" t="b">
         <v>1</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -899,34 +1007,46 @@
         <v>256GB</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>6.7" Super AMOLED (FHD+ 1080×2340), 90Hz</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>MediaTek Helio G99 (6nm)</v>
       </c>
       <c r="J10" t="str">
         <v>8GB</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>Trasera: 50MP + 5MP ultra gran angular + 2MP macro; Frontal: 13MP</v>
       </c>
       <c r="L10" t="str">
-        <v/>
-      </c>
-      <c r="M10" t="str">
-        <v/>
+        <v>5000mAh, 25W carga</v>
+      </c>
+      <c r="M10">
+        <v>2024</v>
       </c>
       <c r="N10" t="str">
-        <v/>
+        <v>De gama media Samsung teléfono con AMOLED pantalla, Helio G99 chipset, y triple cámaras; soporte de software prolongado.</v>
       </c>
       <c r="O10" t="str">
-        <v/>
+        <v>/images/fotos/p-9.webp</v>
       </c>
       <c r="P10" t="b">
         <v>0</v>
       </c>
       <c r="Q10" t="b">
         <v>1</v>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -952,34 +1072,46 @@
         <v>256GB</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>6.7" Super AMOLED (FHD+ 1080×2340), 120Hz</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>Samsung Exynos 1380 (5nm)</v>
       </c>
       <c r="J11" t="str">
         <v>8GB</v>
       </c>
       <c r="K11" t="str">
-        <v/>
+        <v>Trasera: 50MP + 8MP ultra gran angular + 2MP macro (OIS principal); Frontal: 13MP</v>
       </c>
       <c r="L11" t="str">
-        <v/>
-      </c>
-      <c r="M11" t="str">
-        <v/>
+        <v>5000mAh, 25W carga</v>
+      </c>
+      <c r="M11">
+        <v>2025</v>
       </c>
       <c r="N11" t="str">
-        <v/>
+        <v>Upper De gama media Galaxy A series teléfono con 120Hz AMOLED, Exynos 1380, OIS principal cámara, y 5000mAh batería.</v>
       </c>
       <c r="O11" t="str">
-        <v/>
+        <v>/images/fotos/p-10.webp</v>
       </c>
       <c r="P11" t="b">
         <v>0</v>
       </c>
       <c r="Q11" t="b">
         <v>1</v>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1005,34 +1137,46 @@
         <v>128GB</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>6.7" Super AMOLED (FHD+ 1080×2340), 90Hz</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>Samsung Exynos 1330 (5nm)</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>Trasera: 50MP (OIS) + 5MP ultra gran angular + 2MP macro; Frontal: 13MP</v>
       </c>
       <c r="L12" t="str">
-        <v/>
-      </c>
-      <c r="M12" t="str">
-        <v/>
+        <v>5000mAh, 25W carga rápida</v>
+      </c>
+      <c r="M12">
+        <v>2025</v>
       </c>
       <c r="N12" t="str">
-        <v/>
+        <v>De entrada 5G Galaxy A series teléfono con a 6.7" AMOLED 90Hz pantalla, OIS principal cámara, y soporte de software prolongado.</v>
       </c>
       <c r="O12" t="str">
-        <v/>
+        <v>/images/fotos/p-11.jpg</v>
       </c>
       <c r="P12" t="b">
         <v>0</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1058,34 +1202,46 @@
         <v>128GB</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>6.5" PLS LCD (HD+ 720×1600)</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>Samsung Exynos 850</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K13" t="str">
-        <v/>
+        <v>Trasera: 50MP + 2MP profundidad; Frontal: 5MP</v>
       </c>
       <c r="L13" t="str">
-        <v/>
-      </c>
-      <c r="M13" t="str">
-        <v/>
+        <v>5000mAh</v>
+      </c>
+      <c r="M13">
+        <v>2022</v>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>De entrada Galaxy A teléfono con 6.5" HD+ pantalla, 50MP principal cámara, y 5000mAh batería.</v>
       </c>
       <c r="O13" t="str">
-        <v/>
+        <v>/images/fotos/p-12.png</v>
       </c>
       <c r="P13" t="b">
         <v>0</v>
       </c>
       <c r="Q13" t="b">
         <v>1</v>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1111,34 +1267,46 @@
         <v/>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>6.5" Super AMOLED (FHD+ 1080×2340), 90Hz</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>MediaTek Helio G99 (6nm)</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>4GB / 8GB (varies by version)</v>
       </c>
       <c r="K14" t="str">
-        <v/>
+        <v>Trasera: 50MP + 5MP ultra gran angular + 2MP macro; Frontal: 13MP</v>
       </c>
       <c r="L14" t="str">
-        <v/>
-      </c>
-      <c r="M14" t="str">
-        <v/>
+        <v>5000mAh, 25W carga rápida</v>
+      </c>
+      <c r="M14">
+        <v>2023</v>
       </c>
       <c r="N14" t="str">
-        <v/>
+        <v>Económico Samsung teléfono con an AMOLED 90Hz pantalla, sólida batería life, y a versátil triple-cámara setup.</v>
       </c>
       <c r="O14" t="str">
-        <v/>
+        <v>/images/fotos/p-13.jpg</v>
       </c>
       <c r="P14" t="b">
         <v>0</v>
       </c>
       <c r="Q14" t="b">
         <v>1</v>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1164,34 +1332,46 @@
         <v>256GB</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>6.56" IPS LCD (HD+ 720×1612), 90Hz</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>MediaTek Helio G85</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>8GB (+ up to 8GB extended)</v>
       </c>
       <c r="K15" t="str">
-        <v/>
+        <v>Trasera: 50MP principal; Frontal: 32MP</v>
       </c>
       <c r="L15" t="str">
-        <v/>
-      </c>
-      <c r="M15" t="str">
-        <v/>
+        <v>5000mAh, 18W carga rápida</v>
+      </c>
+      <c r="M15">
+        <v>2023</v>
       </c>
       <c r="N15" t="str">
-        <v/>
+        <v>buena relación calidad-precio-focused Tecno teléfono con Helio G85 rendimiento, 8GB RAM (más memory expansion), y a 50MP cámara.</v>
       </c>
       <c r="O15" t="str">
-        <v/>
+        <v>/images/fotos/p-14.jpg</v>
       </c>
       <c r="P15" t="b">
         <v>0</v>
       </c>
       <c r="Q15" t="b">
         <v>1</v>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1217,34 +1397,46 @@
         <v>256GB</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+ 2400×1080), 120Hz</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>MediaTek Dimensity 7300 Ultra (4nm)</v>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K16" t="str">
-        <v/>
+        <v>Trasera: 200MP (OIS) + 8MP ultra gran angular + 2MP macro; Frontal: 20MP</v>
       </c>
       <c r="L16" t="str">
-        <v/>
-      </c>
-      <c r="M16" t="str">
-        <v/>
+        <v>5110mAh, 45W carga rápida</v>
+      </c>
+      <c r="M16">
+        <v>2024</v>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>Upper De gama media Redmi Note con brillante 120Hz AMOLED pantalla, Dimensity 7300 Ultra rendimiento, y a 200MP OIS principal cámara.</v>
       </c>
       <c r="O16" t="str">
-        <v/>
+        <v>/images/fotos/p-15.jpg</v>
       </c>
       <c r="P16" t="b">
         <v>0</v>
       </c>
       <c r="Q16" t="b">
         <v>1</v>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1270,34 +1462,46 @@
         <v/>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>6.7" Super AMOLED (FHD+ 1080×2340), 90Hz</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>MediaTek Helio G99 (6nm)</v>
       </c>
       <c r="J17" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K17" t="str">
-        <v/>
+        <v>Trasera: 50MP + 5MP ultra gran angular + 2MP macro; Frontal: 13MP</v>
       </c>
       <c r="L17" t="str">
-        <v/>
-      </c>
-      <c r="M17" t="str">
-        <v/>
+        <v>5000mAh, 25W carga</v>
+      </c>
+      <c r="M17">
+        <v>2024</v>
       </c>
       <c r="N17" t="str">
-        <v/>
+        <v>Galaxy A-series De gama media teléfono (SWAP/reacondicionado) con gran AMOLED pantalla, Helio G99 chipset, y long batería life.</v>
       </c>
       <c r="O17" t="str">
-        <v/>
+        <v>/images/fotos/p-16.webp</v>
       </c>
       <c r="P17" t="b">
         <v>0</v>
       </c>
       <c r="Q17" t="b">
         <v>1</v>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1323,34 +1527,46 @@
         <v>128GB</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>6.1" Liquid Retina IPS LCD (1792×828)</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>Apple A13 Bionic</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K18" t="str">
-        <v/>
+        <v>Trasera: 12MP gran angular + 12MP ultra gran angular; Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L18" t="str">
-        <v/>
-      </c>
-      <c r="M18" t="str">
-        <v/>
+        <v>3110mAh (aprox.), carga rápida; Qi inalámbrica</v>
+      </c>
+      <c r="M18">
+        <v>2019</v>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>iPhone 11 (usado/reacondicionado) con A13 Bionic, doble 12MP cámaras, y 6.1" Liquid Retina pantalla.</v>
       </c>
       <c r="O18" t="str">
-        <v/>
+        <v>/images/fotos/p-17.jpg</v>
       </c>
       <c r="P18" t="b">
         <v>0</v>
       </c>
       <c r="Q18" t="b">
         <v>1</v>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1376,34 +1592,46 @@
         <v>128GB</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>6.1" Liquid Retina IPS LCD (1792×828)</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>Apple A12 Bionic</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>3GB</v>
       </c>
       <c r="K19" t="str">
-        <v/>
+        <v>Trasera: 12MP gran angular; Frontal: 7MP TrueDepth</v>
       </c>
       <c r="L19" t="str">
-        <v/>
-      </c>
-      <c r="M19" t="str">
-        <v/>
+        <v>2942mAh (aprox.), carga rápida; Qi inalámbrica</v>
+      </c>
+      <c r="M19">
+        <v>2018</v>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>iPhone XR con A12 Bionic, 6.1" Liquid Retina pantalla, y reliable single-sistema de cámaras.</v>
       </c>
       <c r="O19" t="str">
-        <v/>
+        <v>/images/fotos/p-18.jpeg</v>
       </c>
       <c r="P19" t="b">
         <v>0</v>
       </c>
       <c r="Q19" t="b">
         <v>1</v>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1429,34 +1657,46 @@
         <v/>
       </c>
       <c r="H20" t="str">
-        <v/>
+        <v>1.8" TFT</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>Unisoc 6531F (feature phone)</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>4MB</v>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>No camera</v>
       </c>
       <c r="L20" t="str">
-        <v/>
-      </c>
-      <c r="M20" t="str">
-        <v/>
+        <v>800mAh</v>
+      </c>
+      <c r="M20">
+        <v>2018</v>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>Basic feature teléfono focused on calls y SMS con long standby time y a compacto 1.8" pantalla.</v>
       </c>
       <c r="O20" t="str">
-        <v/>
+        <v>/images/fotos/p-19.webp</v>
       </c>
       <c r="P20" t="b">
         <v>0</v>
       </c>
       <c r="Q20" t="b">
         <v>1</v>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1482,34 +1722,46 @@
         <v>64GB</v>
       </c>
       <c r="H21" t="str">
-        <v/>
+        <v>5.8" Super Retina XDR OLED (2436×1125)</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>Apple A13 Bionic</v>
       </c>
       <c r="J21" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K21" t="str">
-        <v/>
+        <v>Trasera: 12MP gran angular + 12MP ultra gran angular + 12MP teleobjetivo; Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L21" t="str">
-        <v/>
-      </c>
-      <c r="M21" t="str">
-        <v/>
+        <v>3046mAh (aprox.), carga rápida; Qi inalámbrica</v>
+      </c>
+      <c r="M21">
+        <v>2019</v>
       </c>
       <c r="N21" t="str">
-        <v/>
+        <v>iPhone 11 Pro (usado/reacondicionado) con triple-sistema de cámaras, OLED pantalla, y A13 Bionic rendimiento.</v>
       </c>
       <c r="O21" t="str">
-        <v/>
+        <v>/images/fotos/p-20.jpg</v>
       </c>
       <c r="P21" t="b">
         <v>0</v>
       </c>
       <c r="Q21" t="b">
         <v>1</v>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1535,34 +1787,46 @@
         <v/>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>6.7" Super AMOLED Plus (FHD+ 1080×2400), 60Hz</v>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 865+ (7nm+) / Exynos 990 (7nm+)</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K22" t="str">
-        <v/>
+        <v>Trasera: 12MP gran angular + 64MP teleobjetivo + 12MP ultra gran angular; Frontal: 10MP</v>
       </c>
       <c r="L22" t="str">
-        <v/>
-      </c>
-      <c r="M22" t="str">
-        <v/>
+        <v>4300mAh, 25W carga rápida; carga inalámbrica</v>
+      </c>
+      <c r="M22">
+        <v>2020</v>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>Premium Samsung tope de gama (SWAP/reacondicionado) con S Pen support, powerful 5G rendimiento, y a versátil triple-sistema de cámaras.</v>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>/images/fotos/p-21.webp</v>
       </c>
       <c r="P22" t="b">
         <v>0</v>
       </c>
       <c r="Q22" t="b">
         <v>1</v>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1588,34 +1852,46 @@
         <v>64GB</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>6.6" PLS LCD (FHD+ 1080×2408)</v>
       </c>
       <c r="I23" t="str">
-        <v/>
+        <v>Samsung Exynos 850 (8nm)</v>
       </c>
       <c r="J23" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K23" t="str">
-        <v/>
+        <v>Trasera: 50MP + 5MP ultra gran angular + 2MP macro + 2MP profundidad; Frontal: 8MP</v>
       </c>
       <c r="L23" t="str">
-        <v/>
-      </c>
-      <c r="M23" t="str">
-        <v/>
+        <v>5000mAh, 15W carga</v>
+      </c>
+      <c r="M23">
+        <v>2022</v>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>De entrada Samsung teléfono con gran FHD+ screen, 50MP principal cámara, y a 5000mAh batería.</v>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>/images/fotos/p-22.jpg</v>
       </c>
       <c r="P23" t="b">
         <v>0</v>
       </c>
       <c r="Q23" t="b">
         <v>1</v>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1641,34 +1917,46 @@
         <v>128GB</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>6.6" IPS LCD (HD+), 90Hz</v>
       </c>
       <c r="I24" t="str">
-        <v/>
+        <v>MediaTek Helio G37</v>
       </c>
       <c r="J24" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K24" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + profundidad; Frontal: 8MP</v>
       </c>
       <c r="L24" t="str">
-        <v/>
-      </c>
-      <c r="M24" t="str">
-        <v/>
+        <v>5000mAh, 18W carga rápida</v>
+      </c>
+      <c r="M24">
+        <v>2023</v>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>Económico Tecno Spark series teléfono con a 90Hz pantalla, Helio G37 chipset, y a 50MP principal cámara.</v>
       </c>
       <c r="O24" t="str">
-        <v/>
+        <v>/images/fotos/p-23.webp</v>
       </c>
       <c r="P24" t="b">
         <v>0</v>
       </c>
       <c r="Q24" t="b">
         <v>1</v>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1694,34 +1982,46 @@
         <v/>
       </c>
       <c r="H25" t="str">
-        <v/>
+        <v>2.4" TFT</v>
       </c>
       <c r="I25" t="str">
-        <v/>
+        <v>Feature phone chipset</v>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>32MB</v>
       </c>
       <c r="K25" t="str">
-        <v/>
+        <v>No camera</v>
       </c>
       <c r="L25" t="str">
-        <v/>
-      </c>
-      <c r="M25" t="str">
-        <v/>
+        <v>1000mAh</v>
+      </c>
+      <c r="M25">
+        <v>2015</v>
       </c>
       <c r="N25" t="str">
-        <v/>
+        <v>Simple feature teléfono for calls y SMS con long standby time y doble-SIM support.</v>
       </c>
       <c r="O25" t="str">
-        <v/>
+        <v>/images/fotos/p-24.webp</v>
       </c>
       <c r="P25" t="b">
         <v>0</v>
       </c>
       <c r="Q25" t="b">
         <v>1</v>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v/>
+      </c>
+      <c r="U25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1747,34 +2047,46 @@
         <v>128GB</v>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>6.56" TFT LCD (HD+ 720×1612), 90Hz</v>
       </c>
       <c r="I26" t="str">
-        <v/>
+        <v>MediaTek Helio G36</v>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K26" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + profundidad; Frontal: 5MP</v>
       </c>
       <c r="L26" t="str">
-        <v/>
-      </c>
-      <c r="M26" t="str">
-        <v/>
+        <v>5200mAh</v>
+      </c>
+      <c r="M26">
+        <v>2024</v>
       </c>
       <c r="N26" t="str">
-        <v/>
+        <v>Económico Honor teléfono con a fluida 90Hz pantalla, 50MP principal cámara, y a gran 5200mAh batería.</v>
       </c>
       <c r="O26" t="str">
-        <v/>
+        <v>/images/fotos/p-25.jpg</v>
       </c>
       <c r="P26" t="b">
         <v>0</v>
       </c>
       <c r="Q26" t="b">
         <v>1</v>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1800,34 +2112,46 @@
         <v>256GB</v>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>6.9" IPS LCD (HD+ 1600×720), hasta 120Hz</v>
       </c>
       <c r="I27" t="str">
-        <v/>
+        <v>MediaTek Dimensity 6300 (6nm)</v>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + auxiliar; Frontal: 8MP</v>
       </c>
       <c r="L27" t="str">
-        <v/>
-      </c>
-      <c r="M27" t="str">
-        <v/>
+        <v>6000mAh, 33W carga rápida</v>
+      </c>
+      <c r="M27">
+        <v>2025</v>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>Económico 5G teléfono con gran 6.9" 120Hz pantalla, Dimensity 6300 rendimiento, y a 6000mAh batería; incluye Xiaomi HyperOS.</v>
       </c>
       <c r="O27" t="str">
-        <v/>
+        <v>/images/fotos/p-26.jpg</v>
       </c>
       <c r="P27" t="b">
         <v>0</v>
       </c>
       <c r="Q27" t="b">
         <v>1</v>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1853,34 +2177,46 @@
         <v>64GB</v>
       </c>
       <c r="H28" t="str">
-        <v/>
+        <v>6.7" PLS LCD (HD+ 720×1600)</v>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>MediaTek Helio G85 (12nm)</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K28" t="str">
-        <v/>
+        <v>Trasera: 50MP + 2MP profundidad; Frontal: 8MP</v>
       </c>
       <c r="L28" t="str">
-        <v/>
-      </c>
-      <c r="M28" t="str">
-        <v/>
+        <v>5000mAh, 25W carga</v>
+      </c>
+      <c r="M28">
+        <v>2024</v>
       </c>
       <c r="N28" t="str">
-        <v/>
+        <v>De entrada Samsung teléfono con gran 6.7" pantalla, Helio G85 rendimiento, y 5000mAh batería.</v>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>/images/fotos/p-27.jpg</v>
       </c>
       <c r="P28" t="b">
         <v>0</v>
       </c>
       <c r="Q28" t="b">
         <v>1</v>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1906,34 +2242,46 @@
         <v>128GB</v>
       </c>
       <c r="H29" t="str">
-        <v/>
+        <v>6.7" Super AMOLED (FHD+ 1080×2340), 90Hz</v>
       </c>
       <c r="I29" t="str">
-        <v/>
+        <v>MediaTek Helio G99 (6nm)</v>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>6GB</v>
       </c>
       <c r="K29" t="str">
-        <v/>
+        <v>Trasera: 50MP + 5MP ultra gran angular + 2MP macro; Frontal: 13MP</v>
       </c>
       <c r="L29" t="str">
-        <v/>
-      </c>
-      <c r="M29" t="str">
-        <v/>
+        <v>5000mAh, 25W carga</v>
+      </c>
+      <c r="M29">
+        <v>2024</v>
       </c>
       <c r="N29" t="str">
-        <v/>
+        <v>De gama media Samsung teléfono con AMOLED pantalla, Helio G99 chipset, y triple cámaras; soporte de software prolongado.</v>
       </c>
       <c r="O29" t="str">
-        <v/>
+        <v>/images/fotos/p-28.jpg</v>
       </c>
       <c r="P29" t="b">
         <v>0</v>
       </c>
       <c r="Q29" t="b">
         <v>1</v>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1959,34 +2307,46 @@
         <v/>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>6.7" Dynamic AMOLED 2X (FHD+), 120Hz</v>
       </c>
       <c r="I30" t="str">
-        <v/>
+        <v>Samsung Exynos 2400e</v>
       </c>
       <c r="J30" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>Trasera: 50MP (OIS) + 8MP teleobjetivo (3x) + 12MP ultra gran angular; Frontal: 10MP</v>
       </c>
       <c r="L30" t="str">
-        <v/>
-      </c>
-      <c r="M30" t="str">
-        <v/>
+        <v>4700mAh, 25W carga rápida; carga inalámbrica</v>
+      </c>
+      <c r="M30">
+        <v>2024</v>
       </c>
       <c r="N30" t="str">
-        <v/>
+        <v>Fan Edition tope de gama con a 120Hz AMOLED pantalla, tope de gama-class rendimiento, y a versátil sistema de cámaras con 3x teleobjetivo.</v>
       </c>
       <c r="O30" t="str">
-        <v/>
+        <v>/images/fotos/p-29.jpg</v>
       </c>
       <c r="P30" t="b">
         <v>0</v>
       </c>
       <c r="Q30" t="b">
         <v>1</v>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
+      <c r="S30" t="str">
+        <v/>
+      </c>
+      <c r="T30" t="str">
+        <v/>
+      </c>
+      <c r="U30" t="str">
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -2012,34 +2372,46 @@
         <v/>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>6.4" Dynamic AMOLED 2X (FHD+), 120Hz</v>
       </c>
       <c r="I31" t="str">
-        <v/>
+        <v>Samsung Exynos 2200 / Qualcomm Snapdragon 8 Gen 1</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K31" t="str">
-        <v/>
+        <v>Trasera: 50MP (OIS) + 8MP teleobjetivo (3x) + 12MP ultra gran angular; Frontal: 10MP</v>
       </c>
       <c r="L31" t="str">
-        <v/>
-      </c>
-      <c r="M31" t="str">
-        <v/>
+        <v>4500mAh, 25W carga rápida; carga inalámbrica</v>
+      </c>
+      <c r="M31">
+        <v>2023</v>
       </c>
       <c r="N31" t="str">
-        <v/>
+        <v>Fan Edition tope de gama (SWAP/reacondicionado) con 120Hz AMOLED, strong rendimiento, y teleobjetivo cámara for 3x zoom.</v>
       </c>
       <c r="O31" t="str">
-        <v/>
+        <v>/images/fotos/p-30.webp</v>
       </c>
       <c r="P31" t="b">
         <v>0</v>
       </c>
       <c r="Q31" t="b">
         <v>1</v>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
+      <c r="S31" t="str">
+        <v/>
+      </c>
+      <c r="T31" t="str">
+        <v/>
+      </c>
+      <c r="U31" t="str">
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -2065,34 +2437,46 @@
         <v>128GB</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>6.1" Super Retina XDR OLED (2556×1179)</v>
       </c>
       <c r="I32" t="str">
-        <v/>
+        <v>Apple A16 Bionic</v>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>6GB</v>
       </c>
       <c r="K32" t="str">
-        <v/>
+        <v>Trasera: 48MP gran angular + 12MP ultra gran angular; Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L32" t="str">
-        <v/>
-      </c>
-      <c r="M32" t="str">
-        <v/>
+        <v>3349mAh (aprox.), carga rápida; MagSafe inalámbrica</v>
+      </c>
+      <c r="M32">
+        <v>2023</v>
       </c>
       <c r="N32" t="str">
-        <v/>
+        <v>iPhone 15 (SWAP/reacondicionado) con A16 Bionic, 48MP principal cámara, y a 6.1" OLED pantalla.</v>
       </c>
       <c r="O32" t="str">
-        <v/>
+        <v>/images/fotos/p-31.webp</v>
       </c>
       <c r="P32" t="b">
         <v>0</v>
       </c>
       <c r="Q32" t="b">
         <v>1</v>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
+        <v/>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -2118,34 +2502,46 @@
         <v>128GB</v>
       </c>
       <c r="H33" t="str">
-        <v/>
+        <v>6.1" Super Retina XDR OLED (2532×1170)</v>
       </c>
       <c r="I33" t="str">
-        <v/>
+        <v>Apple A14 Bionic</v>
       </c>
       <c r="J33" t="str">
-        <v/>
+        <v>4GB</v>
       </c>
       <c r="K33" t="str">
-        <v/>
+        <v>Trasera: 12MP gran angular + 12MP ultra gran angular; Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L33" t="str">
-        <v/>
-      </c>
-      <c r="M33" t="str">
-        <v/>
+        <v>2815mAh (aprox.), carga rápida; MagSafe inalámbrica</v>
+      </c>
+      <c r="M33">
+        <v>2020</v>
       </c>
       <c r="N33" t="str">
-        <v/>
+        <v>iPhone 12 (SWAP/reacondicionado) con 5G, A14 Bionic, OLED pantalla, y doble 12MP cámaras.</v>
       </c>
       <c r="O33" t="str">
-        <v/>
+        <v>/images/fotos/p-32.jpg</v>
       </c>
       <c r="P33" t="b">
         <v>0</v>
       </c>
       <c r="Q33" t="b">
         <v>1</v>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -2171,34 +2567,46 @@
         <v>128GB</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>6.1" Super Retina XDR OLED (2532×1170), 120Hz (ProMotion)</v>
       </c>
       <c r="I34" t="str">
-        <v/>
+        <v>Apple A15 Bionic</v>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>6GB</v>
       </c>
       <c r="K34" t="str">
-        <v/>
+        <v>Trasera: 12MP gran angular + 12MP ultra gran angular + 12MP teleobjetivo (3x); Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L34" t="str">
-        <v/>
-      </c>
-      <c r="M34" t="str">
-        <v/>
+        <v>3095mAh (aprox.), carga rápida; MagSafe inalámbrica</v>
+      </c>
+      <c r="M34">
+        <v>2021</v>
       </c>
       <c r="N34" t="str">
-        <v/>
+        <v>iPhone 13 Pro (SWAP/reacondicionado) con ProMotion 120Hz pantalla y triple-sistema de cámaras con 3x optical zoom.</v>
       </c>
       <c r="O34" t="str">
-        <v/>
+        <v>/images/fotos/p-33.jpg</v>
       </c>
       <c r="P34" t="b">
         <v>0</v>
       </c>
       <c r="Q34" t="b">
         <v>1</v>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -2224,34 +2632,46 @@
         <v>256GB</v>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>6.1" Super Retina XDR OLED (2556×1179), 120Hz (ProMotion)</v>
       </c>
       <c r="I35" t="str">
-        <v/>
+        <v>Apple A16 Bionic</v>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>6GB</v>
       </c>
       <c r="K35" t="str">
-        <v/>
+        <v>Trasera: 48MP principal + 12MP ultra gran angular + 12MP teleobjetivo (3x); Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L35" t="str">
-        <v/>
-      </c>
-      <c r="M35" t="str">
-        <v/>
+        <v>3200mAh (aprox.), carga rápida; MagSafe inalámbrica</v>
+      </c>
+      <c r="M35">
+        <v>2022</v>
       </c>
       <c r="N35" t="str">
-        <v/>
+        <v>iPhone 14 Pro (SWAP/reacondicionado) con Dynamic Island, A16 Bionic, y 48MP principal cámara más 3x teleobjetivo.</v>
       </c>
       <c r="O35" t="str">
-        <v/>
+        <v>/images/fotos/p-34.jpg</v>
       </c>
       <c r="P35" t="b">
         <v>0</v>
       </c>
       <c r="Q35" t="b">
         <v>1</v>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -2277,34 +2697,46 @@
         <v>128GB</v>
       </c>
       <c r="H36" t="str">
-        <v/>
+        <v>6.7" Super Retina XDR OLED (2778×1284), 120Hz (ProMotion)</v>
       </c>
       <c r="I36" t="str">
-        <v/>
+        <v>Apple A15 Bionic</v>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>6GB</v>
       </c>
       <c r="K36" t="str">
-        <v/>
+        <v>Trasera: 12MP gran angular + 12MP ultra gran angular + 12MP teleobjetivo (3x); Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L36" t="str">
-        <v/>
-      </c>
-      <c r="M36" t="str">
-        <v/>
+        <v>4352mAh (aprox.), carga rápida; MagSafe inalámbrica</v>
+      </c>
+      <c r="M36">
+        <v>2021</v>
       </c>
       <c r="N36" t="str">
-        <v/>
+        <v>iPhone 13 Pro Max (SWAP/reacondicionado) con gran 6.7" 120Hz pantalla y triple cámaras incluyendo 3x optical zoom.</v>
       </c>
       <c r="O36" t="str">
-        <v/>
+        <v>/images/fotos/p-35.jpg</v>
       </c>
       <c r="P36" t="b">
         <v>0</v>
       </c>
       <c r="Q36" t="b">
         <v>1</v>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
+        <v/>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -2330,34 +2762,46 @@
         <v>256GB</v>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>6.2" Dynamic LTPO AMOLED 2X (FHD+ 2340×1080), 1–120Hz</v>
       </c>
       <c r="I37" t="str">
-        <v/>
+        <v>Snapdragon 8 Elite for Galaxy (3nm)</v>
       </c>
       <c r="J37" t="str">
         <v>12GB</v>
       </c>
       <c r="K37" t="str">
-        <v/>
+        <v>Trasera: 50MP gran angular (OIS) + 12MP ultra gran angular + 10MP teleobjetivo (3x, OIS); Frontal: 12MP</v>
       </c>
       <c r="L37" t="str">
-        <v/>
-      </c>
-      <c r="M37" t="str">
-        <v/>
+        <v>4000mAh, 25W por cable; carga inalámbrica</v>
+      </c>
+      <c r="M37">
+        <v>2025</v>
       </c>
       <c r="N37" t="str">
-        <v/>
+        <v>compacto 2025 Samsung tope de gama con Snapdragon 8 Elite for Galaxy, 120Hz AMOLED pantalla, y triple-sistema de cámaras con 3x teleobjetivo.</v>
       </c>
       <c r="O37" t="str">
-        <v/>
+        <v>/images/fotos/p-36.jpg</v>
       </c>
       <c r="P37" t="b">
         <v>0</v>
       </c>
       <c r="Q37" t="b">
         <v>1</v>
+      </c>
+      <c r="R37" t="str">
+        <v/>
+      </c>
+      <c r="S37" t="str">
+        <v/>
+      </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
+      <c r="U37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -2383,34 +2827,46 @@
         <v>256GB</v>
       </c>
       <c r="H38" t="str">
-        <v/>
+        <v>6.7" Dynamic LTPO AMOLED 2X (QHD+ 3120×1440), 1–120Hz</v>
       </c>
       <c r="I38" t="str">
-        <v/>
+        <v>Snapdragon 8 Elite for Galaxy (3nm)</v>
       </c>
       <c r="J38" t="str">
         <v>12GB</v>
       </c>
       <c r="K38" t="str">
-        <v/>
+        <v>Trasera: 50MP gran angular (OIS) + 12MP ultra gran angular + 10MP teleobjetivo (3x, OIS); Frontal: 12MP</v>
       </c>
       <c r="L38" t="str">
-        <v/>
-      </c>
-      <c r="M38" t="str">
-        <v/>
+        <v>4900mAh, 45W por cable; carga inalámbrica</v>
+      </c>
+      <c r="M38">
+        <v>2025</v>
       </c>
       <c r="N38" t="str">
-        <v/>
+        <v>gran-screen 2025 Samsung tope de gama con QHD+ 120Hz AMOLED, Snapdragon 8 Elite for Galaxy, y a versátil triple-cámara setup.</v>
       </c>
       <c r="O38" t="str">
-        <v/>
+        <v>/images/fotos/p-37.jpg</v>
       </c>
       <c r="P38" t="b">
         <v>0</v>
       </c>
       <c r="Q38" t="b">
         <v>1</v>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -2436,34 +2892,46 @@
         <v>512GB</v>
       </c>
       <c r="H39" t="str">
-        <v/>
+        <v>6.7" Dynamic LTPO AMOLED 2X (QHD+ 3120×1440), 1–120Hz</v>
       </c>
       <c r="I39" t="str">
-        <v/>
+        <v>Snapdragon 8 Elite for Galaxy (3nm)</v>
       </c>
       <c r="J39" t="str">
         <v>12GB</v>
       </c>
       <c r="K39" t="str">
-        <v/>
+        <v>Trasera: 50MP gran angular (OIS) + 12MP ultra gran angular + 10MP teleobjetivo (3x, OIS); Frontal: 12MP</v>
       </c>
       <c r="L39" t="str">
-        <v/>
-      </c>
-      <c r="M39" t="str">
-        <v/>
+        <v>4900mAh, 45W por cable; carga inalámbrica</v>
+      </c>
+      <c r="M39">
+        <v>2025</v>
       </c>
       <c r="N39" t="str">
-        <v/>
+        <v>Galaxy S25+ con 512GB storage: QHD+ 120Hz AMOLED, Snapdragon 8 Elite for Galaxy, y triple rear cámaras con 3x teleobjetivo.</v>
       </c>
       <c r="O39" t="str">
-        <v/>
+        <v>/images/fotos/p-38.jpg</v>
       </c>
       <c r="P39" t="b">
         <v>0</v>
       </c>
       <c r="Q39" t="b">
         <v>1</v>
+      </c>
+      <c r="R39" t="str">
+        <v/>
+      </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -2489,34 +2957,46 @@
         <v>256GB</v>
       </c>
       <c r="H40" t="str">
-        <v/>
+        <v>6.9" Dynamic LTPO AMOLED 2X (QHD+ 3120×1440), 1–120Hz</v>
       </c>
       <c r="I40" t="str">
-        <v/>
+        <v>Snapdragon 8 Elite for Galaxy (3nm)</v>
       </c>
       <c r="J40" t="str">
         <v>12GB</v>
       </c>
       <c r="K40" t="str">
-        <v/>
+        <v>Trasera: 200MP gran angular (OIS) + 50MP periscópico (5x, OIS) + 10MP teleobjetivo (3x, OIS) + 50MP ultra gran angular; Frontal: 12MP</v>
       </c>
       <c r="L40" t="str">
-        <v/>
-      </c>
-      <c r="M40" t="str">
-        <v/>
+        <v>5000mAh, 45W por cable; carga inalámbrica</v>
+      </c>
+      <c r="M40">
+        <v>2025</v>
       </c>
       <c r="N40" t="str">
-        <v/>
+        <v>de primer nivel Samsung tope de gama con S Pen, 6.9" QHD+ 120Hz AMOLED, Snapdragon 8 Elite for Galaxy, y a 200MP quad-sistema de cámaras.</v>
       </c>
       <c r="O40" t="str">
-        <v/>
+        <v>/images/fotos/p-39.jpg</v>
       </c>
       <c r="P40" t="b">
         <v>0</v>
       </c>
       <c r="Q40" t="b">
         <v>1</v>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v/>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -2542,34 +3022,46 @@
         <v>512GB</v>
       </c>
       <c r="H41" t="str">
-        <v/>
+        <v>6.9" Dynamic LTPO AMOLED 2X (QHD+ 3120×1440), 1–120Hz</v>
       </c>
       <c r="I41" t="str">
-        <v/>
+        <v>Snapdragon 8 Elite for Galaxy (3nm)</v>
       </c>
       <c r="J41" t="str">
         <v>12GB</v>
       </c>
       <c r="K41" t="str">
-        <v/>
+        <v>Trasera: 200MP gran angular (OIS) + 50MP periscópico (5x, OIS) + 10MP teleobjetivo (3x, OIS) + 50MP ultra gran angular; Frontal: 12MP</v>
       </c>
       <c r="L41" t="str">
-        <v/>
-      </c>
-      <c r="M41" t="str">
-        <v/>
+        <v>5000mAh, 45W por cable; carga inalámbrica</v>
+      </c>
+      <c r="M41">
+        <v>2025</v>
       </c>
       <c r="N41" t="str">
-        <v/>
+        <v>Galaxy S25 Ultra con 512GB storage: S Pen tope de gama con 200MP quad cámaras, Snapdragon 8 Elite for Galaxy, y long-lasting 5000mAh batería.</v>
       </c>
       <c r="O41" t="str">
-        <v/>
+        <v>/images/fotos/p-40.jpg</v>
       </c>
       <c r="P41" t="b">
         <v>0</v>
       </c>
       <c r="Q41" t="b">
         <v>1</v>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
+      <c r="T41" t="str">
+        <v/>
+      </c>
+      <c r="U41" t="str">
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -2595,34 +3087,46 @@
         <v>256GB</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>6.7" Dynamic AMOLED 2X (FHD+ 2340×1080), 120Hz</v>
       </c>
       <c r="I42" t="str">
-        <v/>
+        <v>Samsung Exynos 2400 (4nm)</v>
       </c>
       <c r="J42" t="str">
         <v>8GB</v>
       </c>
       <c r="K42" t="str">
-        <v/>
+        <v>Trasera: 50MP (OIS) + 12MP ultra gran angular + 8MP teleobjetivo (3x, OIS); Frontal: 12MP</v>
       </c>
       <c r="L42" t="str">
-        <v/>
-      </c>
-      <c r="M42" t="str">
-        <v/>
+        <v>4900mAh, 45W por cable; 15W carga inalámbrica</v>
+      </c>
+      <c r="M42">
+        <v>2025</v>
       </c>
       <c r="N42" t="str">
-        <v/>
+        <v>Fan Edition model bringing tope de gama-like Galaxy AI features con a 6.7" 120Hz AMOLED pantalla, Exynos 2400 chipset, y triple cámaras incluyendo 3x teleobjetivo.</v>
       </c>
       <c r="O42" t="str">
-        <v/>
+        <v>/images/fotos/p-41.jpg</v>
       </c>
       <c r="P42" t="b">
         <v>0</v>
       </c>
       <c r="Q42" t="b">
         <v>1</v>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -2648,34 +3152,46 @@
         <v>512GB</v>
       </c>
       <c r="H43" t="str">
-        <v/>
+        <v>6.7" Dynamic AMOLED 2X (FHD+ 2340×1080), 120Hz</v>
       </c>
       <c r="I43" t="str">
-        <v/>
+        <v>Samsung Exynos 2400 (4nm)</v>
       </c>
       <c r="J43" t="str">
         <v>8GB</v>
       </c>
       <c r="K43" t="str">
-        <v/>
+        <v>Trasera: 50MP (OIS) + 12MP ultra gran angular + 8MP teleobjetivo (3x, OIS); Frontal: 12MP</v>
       </c>
       <c r="L43" t="str">
-        <v/>
-      </c>
-      <c r="M43" t="str">
-        <v/>
+        <v>4900mAh, 45W por cable; 15W carga inalámbrica</v>
+      </c>
+      <c r="M43">
+        <v>2025</v>
       </c>
       <c r="N43" t="str">
-        <v/>
+        <v>Galaxy S25 FE con 512GB storage: 6.7" 120Hz AMOLED, Exynos 2400, 3x teleobjetivo cámara, y faster 45W carga.</v>
       </c>
       <c r="O43" t="str">
-        <v/>
+        <v>/images/fotos/p-42.jpg</v>
       </c>
       <c r="P43" t="b">
         <v>0</v>
       </c>
       <c r="Q43" t="b">
         <v>1</v>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -2701,34 +3217,46 @@
         <v>256GB</v>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>6.8" Dynamic LTPO AMOLED 2X (QHD+ 3120×1440), 1–120Hz</v>
       </c>
       <c r="I44" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 8 Gen 3 for Galaxy</v>
       </c>
       <c r="J44" t="str">
         <v>12GB</v>
       </c>
       <c r="K44" t="str">
-        <v/>
+        <v>Trasera: 200MP (OIS) + 50MP periscópico (5x, OIS) + 10MP teleobjetivo (3x, OIS) + 12MP ultra gran angular; Frontal: 12MP</v>
       </c>
       <c r="L44" t="str">
-        <v/>
-      </c>
-      <c r="M44" t="str">
-        <v/>
+        <v>5000mAh, 45W por cable; 15W carga inalámbrica</v>
+      </c>
+      <c r="M44">
+        <v>2024</v>
       </c>
       <c r="N44" t="str">
-        <v/>
+        <v>Samsung’s 2024 Ultra tope de gama con titanium build, S Pen, 200MP principal cámara, y Snapdragon 8 Gen 3 rendimiento.</v>
       </c>
       <c r="O44" t="str">
-        <v/>
+        <v>/images/fotos/p-43.jpg</v>
       </c>
       <c r="P44" t="b">
         <v>0</v>
       </c>
       <c r="Q44" t="b">
         <v>1</v>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+      <c r="S44" t="str">
+        <v/>
+      </c>
+      <c r="T44" t="str">
+        <v/>
+      </c>
+      <c r="U44" t="str">
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -2754,34 +3282,46 @@
         <v>512GB</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>6.8" Dynamic LTPO AMOLED 2X (QHD+ 3120×1440), 1–120Hz</v>
       </c>
       <c r="I45" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 8 Gen 3 for Galaxy</v>
       </c>
       <c r="J45" t="str">
         <v>12GB</v>
       </c>
       <c r="K45" t="str">
-        <v/>
+        <v>Trasera: 200MP (OIS) + 50MP periscópico (5x, OIS) + 10MP teleobjetivo (3x, OIS) + 12MP ultra gran angular; Frontal: 12MP</v>
       </c>
       <c r="L45" t="str">
-        <v/>
-      </c>
-      <c r="M45" t="str">
-        <v/>
+        <v>5000mAh, 45W por cable; 15W carga inalámbrica</v>
+      </c>
+      <c r="M45">
+        <v>2024</v>
       </c>
       <c r="N45" t="str">
-        <v/>
+        <v>Galaxy S24 Ultra con 512GB storage: de primer nivel Android tope de gama con S Pen, 200MP quad cámaras, y a brillante QHD+ 120Hz pantalla.</v>
       </c>
       <c r="O45" t="str">
-        <v/>
+        <v>/images/fotos/p-44.jpg</v>
       </c>
       <c r="P45" t="b">
         <v>0</v>
       </c>
       <c r="Q45" t="b">
         <v>1</v>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v/>
+      </c>
+      <c r="U45" t="str">
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -2807,34 +3347,46 @@
         <v>256GB</v>
       </c>
       <c r="H46" t="str">
-        <v/>
+        <v>6.8" Dynamic AMOLED 2X (QHD+ 3088×1440), 1–120Hz</v>
       </c>
       <c r="I46" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 8 Gen 2 for Galaxy</v>
       </c>
       <c r="J46" t="str">
         <v>12GB</v>
       </c>
       <c r="K46" t="str">
-        <v/>
+        <v>Trasera: 200MP (OIS) + 10MP periscópico (10x, OIS) + 10MP teleobjetivo (3x, OIS) + 12MP ultra gran angular; Frontal: 12MP</v>
       </c>
       <c r="L46" t="str">
-        <v/>
-      </c>
-      <c r="M46" t="str">
-        <v/>
+        <v>5000mAh, 45W por cable; carga inalámbrica</v>
+      </c>
+      <c r="M46">
+        <v>2023</v>
       </c>
       <c r="N46" t="str">
-        <v/>
+        <v>Samsung 2023 Ultra tope de gama con S Pen, Snapdragon 8 Gen 2 for Galaxy, y versátil 200MP quad-cámara setup incluyendo 10x optical zoom.</v>
       </c>
       <c r="O46" t="str">
-        <v/>
+        <v>/images/fotos/p-45.webp</v>
       </c>
       <c r="P46" t="b">
         <v>0</v>
       </c>
       <c r="Q46" t="b">
         <v>1</v>
+      </c>
+      <c r="R46" t="str">
+        <v/>
+      </c>
+      <c r="S46" t="str">
+        <v/>
+      </c>
+      <c r="T46" t="str">
+        <v/>
+      </c>
+      <c r="U46" t="str">
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -2860,34 +3412,46 @@
         <v>128GB</v>
       </c>
       <c r="H47" t="str">
-        <v/>
+        <v>6.3" Super Retina XDR OLED (2622×1206), 1–120Hz (ProMotion)</v>
       </c>
       <c r="I47" t="str">
-        <v/>
+        <v>Apple A18 Pro</v>
       </c>
       <c r="J47" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K47" t="str">
-        <v/>
+        <v>Trasera: 48MP Fusion + 48MP Ultra gran angular + 12MP 5x teleobjetivo; Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L47" t="str">
-        <v/>
-      </c>
-      <c r="M47" t="str">
-        <v/>
+        <v>3582mAh</v>
+      </c>
+      <c r="M47">
+        <v>2024</v>
       </c>
       <c r="N47" t="str">
-        <v/>
+        <v>iPhone 16 Pro (eSIM, SWAP/reacondicionado) con 6.3" 120Hz OLED pantalla, A18 Pro chip, y pro triple-sistema de cámaras incluyendo 5x teleobjetivo.</v>
       </c>
       <c r="O47" t="str">
-        <v/>
+        <v>/images/fotos/p-46.jpg</v>
       </c>
       <c r="P47" t="b">
         <v>0</v>
       </c>
       <c r="Q47" t="b">
         <v>1</v>
+      </c>
+      <c r="R47" t="str">
+        <v/>
+      </c>
+      <c r="S47" t="str">
+        <v/>
+      </c>
+      <c r="T47" t="str">
+        <v/>
+      </c>
+      <c r="U47" t="str">
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -2913,34 +3477,46 @@
         <v>256GB</v>
       </c>
       <c r="H48" t="str">
-        <v/>
+        <v>6.9" Super Retina XDR OLED (2868×1320), 1–120Hz (ProMotion)</v>
       </c>
       <c r="I48" t="str">
-        <v/>
+        <v>Apple A18 Pro</v>
       </c>
       <c r="J48" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K48" t="str">
-        <v/>
+        <v>Trasera: 48MP Fusion + 48MP Ultra gran angular + 12MP 5x teleobjetivo; Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L48" t="str">
-        <v/>
-      </c>
-      <c r="M48" t="str">
-        <v/>
+        <v>4685mAh</v>
+      </c>
+      <c r="M48">
+        <v>2024</v>
       </c>
       <c r="N48" t="str">
-        <v/>
+        <v>iPhone 16 Pro Max (eSIM, SWAP/reacondicionado) con gran 6.9" 120Hz OLED pantalla, A18 Pro chip, y pro sistema de cámaras con 5x teleobjetivo.</v>
       </c>
       <c r="O48" t="str">
-        <v/>
+        <v>/images/fotos/p-47.jpg</v>
       </c>
       <c r="P48" t="b">
         <v>0</v>
       </c>
       <c r="Q48" t="b">
         <v>1</v>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+      <c r="S48" t="str">
+        <v/>
+      </c>
+      <c r="T48" t="str">
+        <v/>
+      </c>
+      <c r="U48" t="str">
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -2966,34 +3542,46 @@
         <v>128GB</v>
       </c>
       <c r="H49" t="str">
-        <v/>
+        <v>6.1" Super Retina XDR OLED (2556×1179), 1–120Hz (ProMotion)</v>
       </c>
       <c r="I49" t="str">
-        <v/>
+        <v>Apple A17 Pro</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K49" t="str">
-        <v/>
+        <v>Trasera: 48MP principal + 12MP ultra gran angular + 12MP teleobjetivo (3x); Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L49" t="str">
-        <v/>
-      </c>
-      <c r="M49" t="str">
-        <v/>
+        <v>3274mAh</v>
+      </c>
+      <c r="M49">
+        <v>2023</v>
       </c>
       <c r="N49" t="str">
-        <v/>
+        <v>iPhone 15 Pro (eSIM, SWAP/reacondicionado) con titanium design, A17 Pro chip, y triple-sistema de cámaras con 3x optical zoom.</v>
       </c>
       <c r="O49" t="str">
-        <v/>
+        <v>/images/fotos/p-48.jpg</v>
       </c>
       <c r="P49" t="b">
         <v>0</v>
       </c>
       <c r="Q49" t="b">
         <v>1</v>
+      </c>
+      <c r="R49" t="str">
+        <v/>
+      </c>
+      <c r="S49" t="str">
+        <v/>
+      </c>
+      <c r="T49" t="str">
+        <v/>
+      </c>
+      <c r="U49" t="str">
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -3019,34 +3607,46 @@
         <v>256GB</v>
       </c>
       <c r="H50" t="str">
-        <v/>
+        <v>6.1" Super Retina XDR OLED (2556×1179), 1–120Hz (ProMotion)</v>
       </c>
       <c r="I50" t="str">
-        <v/>
+        <v>Apple A17 Pro</v>
       </c>
       <c r="J50" t="str">
-        <v/>
+        <v>8GB</v>
       </c>
       <c r="K50" t="str">
-        <v/>
+        <v>Trasera: 48MP principal + 12MP ultra gran angular + 12MP teleobjetivo (3x); Frontal: 12MP TrueDepth</v>
       </c>
       <c r="L50" t="str">
-        <v/>
-      </c>
-      <c r="M50" t="str">
-        <v/>
+        <v>3274mAh</v>
+      </c>
+      <c r="M50">
+        <v>2023</v>
       </c>
       <c r="N50" t="str">
-        <v/>
+        <v>iPhone 15 Pro 256GB (eSIM, SWAP/reacondicionado) con titanium build, A17 Pro rendimiento, y pro cámaras incluyendo 3x teleobjetivo.</v>
       </c>
       <c r="O50" t="str">
-        <v/>
+        <v>/images/fotos/p-49.jpg</v>
       </c>
       <c r="P50" t="b">
         <v>0</v>
       </c>
       <c r="Q50" t="b">
         <v>1</v>
+      </c>
+      <c r="R50" t="str">
+        <v/>
+      </c>
+      <c r="S50" t="str">
+        <v/>
+      </c>
+      <c r="T50" t="str">
+        <v/>
+      </c>
+      <c r="U50" t="str">
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -3072,34 +3672,46 @@
         <v>512GB</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>6.36" LTPO OLED (1200×2670), 1–120Hz</v>
       </c>
       <c r="I51" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 8 Elite</v>
       </c>
       <c r="J51" t="str">
         <v>12GB</v>
       </c>
       <c r="K51" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + 50MP ultra gran angular + 50MP teleobjetivo (3x, Leica); Frontal: 32MP</v>
       </c>
       <c r="L51" t="str">
-        <v/>
-      </c>
-      <c r="M51" t="str">
-        <v/>
+        <v>5240mAh, 90W por cable, 50W inalámbrica</v>
+      </c>
+      <c r="M51">
+        <v>2025</v>
       </c>
       <c r="N51" t="str">
-        <v/>
+        <v>compacto Xiaomi tope de gama con Snapdragon 8 Elite rendimiento, Leica triple 50MP cámaras, y rápida 90W carga.</v>
       </c>
       <c r="O51" t="str">
-        <v/>
+        <v>/images/fotos/p-50.jpg</v>
       </c>
       <c r="P51" t="b">
         <v>0</v>
       </c>
       <c r="Q51" t="b">
         <v>1</v>
+      </c>
+      <c r="R51" t="str">
+        <v/>
+      </c>
+      <c r="S51" t="str">
+        <v/>
+      </c>
+      <c r="T51" t="str">
+        <v/>
+      </c>
+      <c r="U51" t="str">
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -3125,34 +3737,46 @@
         <v>512GB</v>
       </c>
       <c r="H52" t="str">
-        <v/>
+        <v>6.73" LTPO AMOLED (QHD+), 1–120Hz</v>
       </c>
       <c r="I52" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 8 Elite</v>
       </c>
       <c r="J52" t="str">
         <v>16GB</v>
       </c>
       <c r="K52" t="str">
-        <v/>
+        <v>Trasera: 50MP principal (1" sensor, OIS) + 50MP ultra gran angular + 50MP teleobjetivo + 200MP periscópico teleobjetivo; Frontal: 32MP</v>
       </c>
       <c r="L52" t="str">
-        <v/>
-      </c>
-      <c r="M52" t="str">
-        <v/>
+        <v>5500mAh, 90W por cable, 50W inalámbrica</v>
+      </c>
+      <c r="M52">
+        <v>2025</v>
       </c>
       <c r="N52" t="str">
-        <v/>
+        <v>Ultra-premium Xiaomi tope de gama con gran QHD+ 120Hz pantalla, Snapdragon 8 Elite rendimiento, y a pro-grade Leica-style multi-cámara setup.</v>
       </c>
       <c r="O52" t="str">
-        <v/>
+        <v>/images/fotos/p-51.jpg</v>
       </c>
       <c r="P52" t="b">
         <v>0</v>
       </c>
       <c r="Q52" t="b">
         <v>1</v>
+      </c>
+      <c r="R52" t="str">
+        <v/>
+      </c>
+      <c r="S52" t="str">
+        <v/>
+      </c>
+      <c r="T52" t="str">
+        <v/>
+      </c>
+      <c r="U52" t="str">
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -3178,34 +3802,46 @@
         <v>512GB</v>
       </c>
       <c r="H53" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), hasta 144Hz</v>
       </c>
       <c r="I53" t="str">
-        <v/>
+        <v>MediaTek Dimensity 8400</v>
       </c>
       <c r="J53" t="str">
         <v>12GB</v>
       </c>
       <c r="K53" t="str">
-        <v/>
+        <v>Trasera: 50MP principal (OIS) + 13MP ultra gran angular + 50MP teleobjetivo; Frontal: 32MP</v>
       </c>
       <c r="L53" t="str">
-        <v/>
-      </c>
-      <c r="M53" t="str">
-        <v/>
+        <v>5000mAh, 67W carga rápida</v>
+      </c>
+      <c r="M53">
+        <v>2025</v>
       </c>
       <c r="N53" t="str">
-        <v/>
+        <v>High-buena relación calidad-precio Xiaomi T-series teléfono con rápida 144Hz AMOLED pantalla, strong Dimensity rendimiento, y a equilibrado triple-sistema de cámaras.</v>
       </c>
       <c r="O53" t="str">
-        <v/>
+        <v>/images/fotos/p-52.jpg</v>
       </c>
       <c r="P53" t="b">
         <v>0</v>
       </c>
       <c r="Q53" t="b">
         <v>1</v>
+      </c>
+      <c r="R53" t="str">
+        <v/>
+      </c>
+      <c r="S53" t="str">
+        <v/>
+      </c>
+      <c r="T53" t="str">
+        <v/>
+      </c>
+      <c r="U53" t="str">
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -3231,34 +3867,46 @@
         <v>512GB</v>
       </c>
       <c r="H54" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), hasta 144Hz</v>
       </c>
       <c r="I54" t="str">
-        <v/>
+        <v>MediaTek Dimensity 9400</v>
       </c>
       <c r="J54" t="str">
         <v>12GB</v>
       </c>
       <c r="K54" t="str">
-        <v/>
+        <v>Trasera: 50MP principal (OIS) + 50MP ultra gran angular + 50MP teleobjetivo; Frontal: 32MP</v>
       </c>
       <c r="L54" t="str">
-        <v/>
-      </c>
-      <c r="M54" t="str">
-        <v/>
+        <v>5000mAh, 120W por cable, 50W inalámbrica</v>
+      </c>
+      <c r="M54">
+        <v>2025</v>
       </c>
       <c r="N54" t="str">
-        <v/>
+        <v>Xiaomi 15T Pro focuses on tope de gama rendimiento y carga rápida, pairing a high-refresh AMOLED pantalla con a versátil triple-cámara setup.</v>
       </c>
       <c r="O54" t="str">
-        <v/>
+        <v>/images/fotos/p-53.jpg</v>
       </c>
       <c r="P54" t="b">
         <v>0</v>
       </c>
       <c r="Q54" t="b">
         <v>1</v>
+      </c>
+      <c r="R54" t="str">
+        <v/>
+      </c>
+      <c r="S54" t="str">
+        <v/>
+      </c>
+      <c r="T54" t="str">
+        <v/>
+      </c>
+      <c r="U54" t="str">
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -3284,34 +3932,46 @@
         <v>1024GB</v>
       </c>
       <c r="H55" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), hasta 144Hz</v>
       </c>
       <c r="I55" t="str">
-        <v/>
+        <v>MediaTek Dimensity 9400</v>
       </c>
       <c r="J55" t="str">
         <v>12GB</v>
       </c>
       <c r="K55" t="str">
-        <v/>
+        <v>Trasera: 50MP principal (OIS) + 50MP ultra gran angular + 50MP teleobjetivo; Frontal: 32MP</v>
       </c>
       <c r="L55" t="str">
-        <v/>
-      </c>
-      <c r="M55" t="str">
-        <v/>
+        <v>5000mAh, 120W por cable, 50W inalámbrica</v>
+      </c>
+      <c r="M55">
+        <v>2025</v>
       </c>
       <c r="N55" t="str">
-        <v/>
+        <v>Xiaomi 15T Pro con 1TB storage: tope de gama-class rendimiento, 144Hz AMOLED pantalla, y muy rápida 120W carga.</v>
       </c>
       <c r="O55" t="str">
-        <v/>
+        <v>/images/fotos/p-54.jpg</v>
       </c>
       <c r="P55" t="b">
         <v>0</v>
       </c>
       <c r="Q55" t="b">
         <v>1</v>
+      </c>
+      <c r="R55" t="str">
+        <v/>
+      </c>
+      <c r="S55" t="str">
+        <v/>
+      </c>
+      <c r="T55" t="str">
+        <v/>
+      </c>
+      <c r="U55" t="str">
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -3337,34 +3997,46 @@
         <v>128GB</v>
       </c>
       <c r="H56" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), 120Hz</v>
       </c>
       <c r="I56" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 7s Gen 3</v>
       </c>
       <c r="J56" t="str">
         <v>6GB</v>
       </c>
       <c r="K56" t="str">
-        <v/>
+        <v>Trasera: 108MP principal + 8MP ultra gran angular + 2MP macro; Frontal: 16MP</v>
       </c>
       <c r="L56" t="str">
-        <v/>
-      </c>
-      <c r="M56" t="str">
-        <v/>
+        <v>5110mAh, 45W carga rápida</v>
+      </c>
+      <c r="M56">
+        <v>2025</v>
       </c>
       <c r="N56" t="str">
-        <v/>
+        <v>Redmi Note De gama media teléfono offering a fluida 120Hz AMOLED pantalla, a high-resolution principal cámara, y strong batería life.</v>
       </c>
       <c r="O56" t="str">
-        <v/>
+        <v>/images/fotos/p-55.jpg</v>
       </c>
       <c r="P56" t="b">
         <v>0</v>
       </c>
       <c r="Q56" t="b">
         <v>1</v>
+      </c>
+      <c r="R56" t="str">
+        <v/>
+      </c>
+      <c r="S56" t="str">
+        <v/>
+      </c>
+      <c r="T56" t="str">
+        <v/>
+      </c>
+      <c r="U56" t="str">
+        <v/>
       </c>
     </row>
     <row r="57">
@@ -3390,34 +4062,46 @@
         <v>256GB</v>
       </c>
       <c r="H57" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), 120Hz</v>
       </c>
       <c r="I57" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 7s Gen 3</v>
       </c>
       <c r="J57" t="str">
         <v>8GB</v>
       </c>
       <c r="K57" t="str">
-        <v/>
+        <v>Trasera: 108MP principal + 8MP ultra gran angular + 2MP macro; Frontal: 16MP</v>
       </c>
       <c r="L57" t="str">
-        <v/>
-      </c>
-      <c r="M57" t="str">
-        <v/>
+        <v>5110mAh, 45W carga rápida</v>
+      </c>
+      <c r="M57">
+        <v>2025</v>
       </c>
       <c r="N57" t="str">
-        <v/>
+        <v>Redmi Note De gama media teléfono con 8GB RAM, 120Hz AMOLED pantalla, y a high-resolution 108MP principal cámara.</v>
       </c>
       <c r="O57" t="str">
-        <v/>
+        <v>/images/fotos/p-56.jpg</v>
       </c>
       <c r="P57" t="b">
         <v>0</v>
       </c>
       <c r="Q57" t="b">
         <v>1</v>
+      </c>
+      <c r="R57" t="str">
+        <v/>
+      </c>
+      <c r="S57" t="str">
+        <v/>
+      </c>
+      <c r="T57" t="str">
+        <v/>
+      </c>
+      <c r="U57" t="str">
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -3443,34 +4127,46 @@
         <v>256GB</v>
       </c>
       <c r="H58" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), 120Hz</v>
       </c>
       <c r="I58" t="str">
-        <v/>
+        <v>MediaTek Dimensity 7300</v>
       </c>
       <c r="J58" t="str">
         <v>8GB</v>
       </c>
       <c r="K58" t="str">
-        <v/>
+        <v>Trasera: 108MP principal (OIS) + 8MP ultra gran angular + 2MP macro; Frontal: 16MP</v>
       </c>
       <c r="L58" t="str">
-        <v/>
-      </c>
-      <c r="M58" t="str">
-        <v/>
+        <v>5110mAh, 67W carga rápida</v>
+      </c>
+      <c r="M58">
+        <v>2025</v>
       </c>
       <c r="N58" t="str">
-        <v/>
+        <v>5G version of Redmi Note con Dimensity rendimiento, fluida 120Hz AMOLED pantalla, y strong batería life con faster carga.</v>
       </c>
       <c r="O58" t="str">
-        <v/>
+        <v>/images/fotos/p-57.jpg</v>
       </c>
       <c r="P58" t="b">
         <v>0</v>
       </c>
       <c r="Q58" t="b">
         <v>1</v>
+      </c>
+      <c r="R58" t="str">
+        <v/>
+      </c>
+      <c r="S58" t="str">
+        <v/>
+      </c>
+      <c r="T58" t="str">
+        <v/>
+      </c>
+      <c r="U58" t="str">
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -3496,34 +4192,46 @@
         <v>256GB</v>
       </c>
       <c r="H59" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), 120Hz</v>
       </c>
       <c r="I59" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 7+ Gen 3</v>
       </c>
       <c r="J59" t="str">
         <v>8GB</v>
       </c>
       <c r="K59" t="str">
-        <v/>
+        <v>Trasera: 200MP (OIS) + 8MP ultra gran angular + 2MP macro; Frontal: 20MP</v>
       </c>
       <c r="L59" t="str">
-        <v/>
-      </c>
-      <c r="M59" t="str">
-        <v/>
+        <v>5110mAh, 67W carga rápida</v>
+      </c>
+      <c r="M59">
+        <v>2025</v>
       </c>
       <c r="N59" t="str">
-        <v/>
+        <v>Redmi Note Pro model con upgraded rendimiento y a high-resolution 200MP OIS principal cámara paired con 120Hz AMOLED.</v>
       </c>
       <c r="O59" t="str">
-        <v/>
+        <v>/images/fotos/p-58.jpg</v>
       </c>
       <c r="P59" t="b">
         <v>0</v>
       </c>
       <c r="Q59" t="b">
         <v>1</v>
+      </c>
+      <c r="R59" t="str">
+        <v/>
+      </c>
+      <c r="S59" t="str">
+        <v/>
+      </c>
+      <c r="T59" t="str">
+        <v/>
+      </c>
+      <c r="U59" t="str">
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -3549,34 +4257,46 @@
         <v>256GB</v>
       </c>
       <c r="H60" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), 120Hz</v>
       </c>
       <c r="I60" t="str">
-        <v/>
+        <v>MediaTek Dimensity 8300</v>
       </c>
       <c r="J60" t="str">
         <v>8GB</v>
       </c>
       <c r="K60" t="str">
-        <v/>
+        <v>Trasera: 200MP (OIS) + 8MP ultra gran angular + 2MP macro; Frontal: 20MP</v>
       </c>
       <c r="L60" t="str">
-        <v/>
-      </c>
-      <c r="M60" t="str">
-        <v/>
+        <v>5110mAh, 67W carga rápida</v>
+      </c>
+      <c r="M60">
+        <v>2025</v>
       </c>
       <c r="N60" t="str">
-        <v/>
+        <v>5G Pro variant con Dimensity chipset, 200MP OIS principal cámara, y fluida 120Hz AMOLED pantalla.</v>
       </c>
       <c r="O60" t="str">
-        <v/>
+        <v>/images/fotos/p-59.jpg</v>
       </c>
       <c r="P60" t="b">
         <v>0</v>
       </c>
       <c r="Q60" t="b">
         <v>1</v>
+      </c>
+      <c r="R60" t="str">
+        <v/>
+      </c>
+      <c r="S60" t="str">
+        <v/>
+      </c>
+      <c r="T60" t="str">
+        <v/>
+      </c>
+      <c r="U60" t="str">
+        <v/>
       </c>
     </row>
     <row r="61">
@@ -3602,34 +4322,46 @@
         <v>512GB</v>
       </c>
       <c r="H61" t="str">
-        <v/>
+        <v>6.67" AMOLED (FHD+), 120Hz</v>
       </c>
       <c r="I61" t="str">
-        <v/>
+        <v>Qualcomm Snapdragon 8s Gen 3</v>
       </c>
       <c r="J61" t="str">
         <v>12GB</v>
       </c>
       <c r="K61" t="str">
-        <v/>
+        <v>Trasera: 200MP (OIS) + 50MP ultra gran angular + 50MP teleobjetivo; Frontal: 20MP</v>
       </c>
       <c r="L61" t="str">
-        <v/>
-      </c>
-      <c r="M61" t="str">
-        <v/>
+        <v>5500mAh, 120W carga rápida</v>
+      </c>
+      <c r="M61">
+        <v>2025</v>
       </c>
       <c r="N61" t="str">
-        <v/>
+        <v>principal Redmi Note Pro+ model con tope de gama-level rendimiento, 200MP OIS cámara, y muy rápida 120W carga.</v>
       </c>
       <c r="O61" t="str">
-        <v/>
+        <v>/images/fotos/p-60.jpg</v>
       </c>
       <c r="P61" t="b">
         <v>0</v>
       </c>
       <c r="Q61" t="b">
         <v>1</v>
+      </c>
+      <c r="R61" t="str">
+        <v/>
+      </c>
+      <c r="S61" t="str">
+        <v/>
+      </c>
+      <c r="T61" t="str">
+        <v/>
+      </c>
+      <c r="U61" t="str">
+        <v/>
       </c>
     </row>
     <row r="62">
@@ -3655,34 +4387,46 @@
         <v>256GB</v>
       </c>
       <c r="H62" t="str">
-        <v/>
+        <v>6.56" TFT LCD (HD+ 720×1612), 90Hz</v>
       </c>
       <c r="I62" t="str">
-        <v/>
+        <v>MediaTek Helio G85</v>
       </c>
       <c r="J62" t="str">
         <v>6GB</v>
       </c>
       <c r="K62" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + profundidad; Frontal: 8MP</v>
       </c>
       <c r="L62" t="str">
-        <v/>
-      </c>
-      <c r="M62" t="str">
-        <v/>
+        <v>5200mAh</v>
+      </c>
+      <c r="M62">
+        <v>2024</v>
       </c>
       <c r="N62" t="str">
-        <v/>
+        <v>Económico Honor teléfono con a fluida 90Hz pantalla, gran batería, y a capable 50MP principal cámara.</v>
       </c>
       <c r="O62" t="str">
-        <v/>
+        <v>/images/fotos/p-61.jpg</v>
       </c>
       <c r="P62" t="b">
         <v>0</v>
       </c>
       <c r="Q62" t="b">
         <v>1</v>
+      </c>
+      <c r="R62" t="str">
+        <v/>
+      </c>
+      <c r="S62" t="str">
+        <v/>
+      </c>
+      <c r="T62" t="str">
+        <v/>
+      </c>
+      <c r="U62" t="str">
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -3708,34 +4452,46 @@
         <v>128GB</v>
       </c>
       <c r="H63" t="str">
-        <v/>
+        <v>6.56" TFT LCD (HD+ 720×1612), 90Hz</v>
       </c>
       <c r="I63" t="str">
-        <v/>
+        <v>MediaTek Helio G36</v>
       </c>
       <c r="J63" t="str">
         <v>4GB</v>
       </c>
       <c r="K63" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + profundidad; Frontal: 5MP</v>
       </c>
       <c r="L63" t="str">
-        <v/>
-      </c>
-      <c r="M63" t="str">
-        <v/>
+        <v>5200mAh</v>
+      </c>
+      <c r="M63">
+        <v>2024</v>
       </c>
       <c r="N63" t="str">
-        <v/>
+        <v>De entrada Honor smartphone con 90Hz pantalla, 50MP principal cámara, y long batería life.</v>
       </c>
       <c r="O63" t="str">
-        <v/>
+        <v>/images/fotos/p-62.jpg</v>
       </c>
       <c r="P63" t="b">
         <v>0</v>
       </c>
       <c r="Q63" t="b">
         <v>1</v>
+      </c>
+      <c r="R63" t="str">
+        <v/>
+      </c>
+      <c r="S63" t="str">
+        <v/>
+      </c>
+      <c r="T63" t="str">
+        <v/>
+      </c>
+      <c r="U63" t="str">
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -3761,34 +4517,46 @@
         <v>128GB</v>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>6.6" IPS LCD (HD+), 90Hz</v>
       </c>
       <c r="I64" t="str">
-        <v/>
+        <v>Unisoc T606</v>
       </c>
       <c r="J64" t="str">
         <v>4GB</v>
       </c>
       <c r="K64" t="str">
-        <v/>
+        <v>Trasera: 50MP principal + 2MP profundidad; Frontal: 8MP</v>
       </c>
       <c r="L64" t="str">
-        <v/>
-      </c>
-      <c r="M64" t="str">
-        <v/>
+        <v>5000mAh, 18W carga</v>
+      </c>
+      <c r="M64">
+        <v>2024</v>
       </c>
       <c r="N64" t="str">
-        <v/>
+        <v>buena relación calidad-precio teléfono con gran pantalla, decent everyday rendimiento, y a gran 5000mAh batería.</v>
       </c>
       <c r="O64" t="str">
-        <v/>
+        <v>/images/fotos/p-63.jpg</v>
       </c>
       <c r="P64" t="b">
         <v>0</v>
       </c>
       <c r="Q64" t="b">
         <v>1</v>
+      </c>
+      <c r="R64" t="str">
+        <v/>
+      </c>
+      <c r="S64" t="str">
+        <v/>
+      </c>
+      <c r="T64" t="str">
+        <v/>
+      </c>
+      <c r="U64" t="str">
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -3814,39 +4582,51 @@
         <v>256GB</v>
       </c>
       <c r="H65" t="str">
-        <v/>
+        <v>6.7" IPS LCD (FHD+), 120Hz</v>
       </c>
       <c r="I65" t="str">
-        <v/>
+        <v>MediaTek Dimensity 7050</v>
       </c>
       <c r="J65" t="str">
         <v>6GB</v>
       </c>
       <c r="K65" t="str">
-        <v/>
+        <v>Trasera: 64MP principal + 8MP ultra gran angular + 2MP macro; Frontal: 16MP</v>
       </c>
       <c r="L65" t="str">
-        <v/>
-      </c>
-      <c r="M65" t="str">
-        <v/>
+        <v>5000mAh, 33W carga rápida</v>
+      </c>
+      <c r="M65">
+        <v>2024</v>
       </c>
       <c r="N65" t="str">
-        <v/>
+        <v>rendimiento-focused Unnecto teléfono con 120Hz pantalla, 5G-capable chipset, y carga rápida.</v>
       </c>
       <c r="O65" t="str">
-        <v/>
+        <v>/images/fotos/p-64.jpg</v>
       </c>
       <c r="P65" t="b">
         <v>0</v>
       </c>
       <c r="Q65" t="b">
         <v>1</v>
+      </c>
+      <c r="R65" t="str">
+        <v/>
+      </c>
+      <c r="S65" t="str">
+        <v/>
+      </c>
+      <c r="T65" t="str">
+        <v/>
+      </c>
+      <c r="U65" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U65"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>